<commit_message>
Importar personal crea sola la estructura que falte (sucursales, departamentos, puestos)
- La validación anuncia «Se creará…» en lugar de marcar error, para quien administra la empresa completa
- Sin duplicados: ignora mayúsculas, acentos y espacios de más; claves cortas automáticas
- Plantilla e instrucciones actualizadas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/usuarios.xlsx
+++ b/public/plantillas/usuarios.xlsx
@@ -69,21 +69,21 @@
     <comment ref="H1" authorId="0">
       <text>
         <r>
-          <t>Opcional. Debe existir en Organización.</t>
+          <t>Opcional. Si no existe en Organización, se crea al importar.</t>
         </r>
       </text>
     </comment>
     <comment ref="I1" authorId="0">
       <text>
         <r>
-          <t>Opcional. Debe existir en Organización. Sirve para asignar cursos por área.</t>
+          <t>Opcional. Si no existe, se crea al importar. Sirve para asignar cursos por área.</t>
         </r>
       </text>
     </comment>
     <comment ref="J1" authorId="0">
       <text>
         <r>
-          <t>Opcional. Debe existir en Organización. Sirve para asignar cursos por puesto.</t>
+          <t>Opcional. Si no existe, se crea al importar. Sirve para asignar cursos por puesto.</t>
         </r>
       </text>
     </comment>
@@ -163,7 +163,7 @@
     <t>2. Cada persona necesita al menos uno de estos tres para poder entrar: Email, Número de empleado o Usuario.</t>
   </si>
   <si>
-    <t>3. Empresa, Sucursal, Departamento y Puesto deben escribirse igual que en la plataforma (Organización).</t>
+    <t>3. La Empresa debe existir en la plataforma. Las sucursales, departamentos y puestos que no existan se crean solos al importar: escríbelos siempre igual (no importan mayúsculas ni acentos).</t>
   </si>
   <si>
     <t>4. Guarda el archivo como Excel (.xlsx) y súbelo en Usuarios → Importar. Antes de crear a nadie, la plataforma revisa todo y marca los errores.</t>
@@ -229,19 +229,19 @@
     <t>ATPVA</t>
   </si>
   <si>
-    <t>Debe existir en Organización.</t>
+    <t>Si no existe en Organización, se crea al importar.</t>
   </si>
   <si>
     <t>Querétaro</t>
   </si>
   <si>
-    <t>Debe existir en Organización. Sirve para asignar cursos por área.</t>
+    <t>Si no existe, se crea al importar. Sirve para asignar cursos por área.</t>
   </si>
   <si>
     <t>Capital Humano</t>
   </si>
   <si>
-    <t>Debe existir en Organización. Sirve para asignar cursos por puesto.</t>
+    <t>Si no existe, se crea al importar. Sirve para asignar cursos por puesto.</t>
   </si>
   <si>
     <t>Analista</t>

</xml_diff>

<commit_message>
Piloto ATPVA: contraseñas que define Capital Humano, visor para celulares viejos y asignaciones sin cuadros repetidos
- Contraseñas: mínimo 6 caracteres; CH puede escribirla (alta, ficha e importación con columna «Contraseña»);
  si no, se crea una fácil («Sol-4827»). Pedir cambio al entrar queda opcional y apagado por omisión.
- Visor de presentaciones: versión «legacy» de pdf.js (fallaba en Chrome 134: Promise.try); si aun así no abre en
  25 s, la lección «Ver todas las páginas» cuenta como vista (evento viewer_failed en bitácora) y se muestra con el
  lector del teléfono. Presentaciones nuevas se completan «Al abrirlas».
- Asignaciones: «Personas específicas» se suma a la asignación activa del curso con las mismas condiciones;
  botón «Agregar personas»; lista agrupada por curso.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/usuarios.xlsx
+++ b/public/plantillas/usuarios.xlsx
@@ -108,12 +108,19 @@
         </r>
       </text>
     </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
+          <t>Opcional. La que Capital Humano le asigna (mínimo 6 caracteres). Si va vacía, la plataforma crea una fácil.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
   <si>
     <t>Nombre</t>
   </si>
@@ -154,6 +161,9 @@
     <t>Fecha de ingreso</t>
   </si>
   <si>
+    <t>Contraseña</t>
+  </si>
+  <si>
     <t>Cómo llenar la plantilla</t>
   </si>
   <si>
@@ -166,7 +176,10 @@
     <t>3. La Empresa debe existir en la plataforma. Las sucursales, departamentos y puestos que no existan se crean solos al importar: escríbelos siempre igual (no importan mayúsculas ni acentos).</t>
   </si>
   <si>
-    <t>4. Guarda el archivo como Excel (.xlsx) y súbelo en Usuarios → Importar. Antes de crear a nadie, la plataforma revisa todo y marca los errores.</t>
+    <t>4. Contraseña: escribe la que le asignas a cada persona (mínimo 6 caracteres) o déjala vacía para que se cree una fácil. Al terminar podrás descargar la lista de accesos.</t>
+  </si>
+  <si>
+    <t>5. Guarda el archivo como Excel (.xlsx) y súbelo en Usuarios → Importar. Antes de crear a nadie, la plataforma revisa todo y marca los errores.</t>
   </si>
   <si>
     <t>Columna</t>
@@ -263,6 +276,12 @@
   </si>
   <si>
     <t>15/01/2024</t>
+  </si>
+  <si>
+    <t>La que Capital Humano le asigna (mínimo 6 caracteres). Si va vacía, la plataforma crea una fácil.</t>
+  </si>
+  <si>
+    <t>Sol-4827</t>
   </si>
 </sst>
 </file>
@@ -680,7 +699,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -694,9 +713,10 @@
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="12" width="14" style="1" customWidth="1"/>
     <col min="13" max="13" width="16" style="2" customWidth="1"/>
+    <col min="14" max="14" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -735,6 +755,9 @@
       </c>
       <c r="M1" s="5" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -746,7 +769,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -757,223 +780,242 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="7" t="s">
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="7" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="B8" s="7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="C8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="B9" s="8" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
+      <c r="C9" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="B10" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B11" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="D11" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B12" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="8" t="s">
+      <c r="C16" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="9" t="s">
+      <c r="C17" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="C18" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+      <c r="B19" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="B20" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>49</v>
+      <c r="B21" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>